<commit_message>
Parts sheet: STEMMA speaker + audio jack pigtail
Rows 22-23: Adafruit STEMMA Speaker #3885 (enclosed class-D amp,
powered from Pmod 3V3, signal from the AUD 3.5 mm jack) and a mono
3.5 mm plug-to-bare-wire pigtail to tap the jack. TOTAL formula
extended to F2:F23.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFCZE5zCJbM3sB1FtBfeBa
</commit_message>
<xml_diff>
--- a/docs/tricorder_parts.xlsx
+++ b/docs/tricorder_parts.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -77,8 +77,11 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <color rgb="000000CC"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +100,11 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0FE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -117,7 +125,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -200,6 +208,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="14" min="1" max="1"/>
@@ -1084,396 +1095,490 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Generic (Amazon)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Dupont jumper wire kit, M-M + M-F + F-F, 10 cm + 20 cm</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" t="n">
+      <c r="D14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="14">
         <f>D14*E14</f>
         <v/>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.com/s?k=dupont+jumper+wire+kit</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="14" t="inlineStr">
         <is>
           <t>Harness for camera, ADC/DAC, mics, AFE control</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="14" t="inlineStr">
         <is>
           <t>Short (10 cm) runs for cam_pclk and adc bus</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Generic (Amazon)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>0.1 in male pin headers, 2x6 Pmod plugs (pack)</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="D15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="14">
         <f>D15*E15</f>
         <v/>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.com/s?k=2x6+pin+header+2.54mm</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>Clean mating into JA/JB/JC/JD/JXADC sockets</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>Alternative: Digilent 2x6 Pmod cable kits</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Adafruit</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>STEMMA QT / Qwiic JST-SH 4-pin cable, 100 mm (#4210)</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="14" t="n">
         <v>0.95</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="14">
         <f>D16*E16</f>
         <v/>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>https://www.adafruit.com/product/4210</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="14" t="inlineStr">
         <is>
           <t>I2C daisy chain across the 5 sensor breakouts</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>Breakouts carry onboard pull-ups; no resistors needed</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="15">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Adafruit</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>JST-SH 4-pin to male dupont adapter cable (#4209)</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
+      <c r="D17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="14" t="n">
         <v>0.95</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="14">
         <f>D17*E17</f>
         <v/>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>https://www.adafruit.com/product/4209</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="14" t="inlineStr">
         <is>
           <t>Qwiic chain entry into Pmod JA1/JA2</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="14" t="inlineStr">
         <is>
           <t>One per harness</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Generic (Amazon)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>SMA male-male cable, RG316, ~30 cm</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" t="n">
+      <c r="D18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="14">
         <f>D18*E18</f>
         <v/>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.com/s?k=sma+male+to+male+rg316</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="14" t="inlineStr">
         <is>
           <t>SiPM eval board to comparator input</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="14" t="inlineStr">
         <is>
           <t>SiPM board is SMA-only</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Generic (Amazon)</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>SMA female pigtail / edge adapter to 0.1 in</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="14">
         <f>D19*E19</f>
         <v/>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.com/s?k=sma+female+pigtail+breadboard</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="14" t="inlineStr">
         <is>
           <t>SiPM comparator + AD8332 analog entries</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="14" t="inlineStr">
         <is>
           <t>One for TLV3501 input, one spare for AFE</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Generic (Amazon)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Solderless breadboard 830pt + wire kit</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="n">
+      <c r="D20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="14">
         <f>D20*E20</f>
         <v/>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.com/s?k=830+breadboard+kit</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="14" t="inlineStr">
         <is>
           <t>TLV3501 comparator, mic-array fan-out, AFE area</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Wiring / connectors</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Generic (Amazon)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Screw terminal block, 2-pin 0.1 in (pack)</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="n">
+      <c r="D21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="14">
         <f>D21*E21</f>
         <v/>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.com/s?k=screw+terminal+2.54mm</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="14" t="inlineStr">
         <is>
           <t>Piezo TX/RX bare-wire attachment</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="14" t="inlineStr">
         <is>
           <t>Twisted pair to the transducers</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Wiring / connectors</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>Adafruit</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>Adafruit STEMMA Speaker #3885 (enclosed, class-D amp, JST-PH)</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F22" s="28">
+        <f>D22*E22</f>
+        <v/>
+      </c>
+      <c r="G22" s="28" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="H22" s="28" t="inlineStr">
+        <is>
+          <t>https://www.adafruit.com/product/3885</t>
+        </is>
+      </c>
+      <c r="I22" s="28" t="inlineStr">
+        <is>
+          <t>Audible scan/alert sounds at the bench</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="inlineStr">
+        <is>
+          <t>Power from Pmod 3V3+GND; signal from the AUD 3.5 mm jack</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="C23" s="25" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="F23" s="26">
-        <f>SUM(F2:F21)</f>
-        <v/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Wiring / connectors</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Generic (Amazon)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3.5 mm mono plug to bare-wire pigtail</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23">
+        <f>D23*E23</f>
+        <v/>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/s?k=3.5mm+mono+plug+pigtail</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Tap the Nexys AUD jack into the STEMMA speaker input</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Mono jack: tip = signal, sleeve = GND</t>
+        </is>
       </c>
     </row>
     <row r="24"/>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="F25" s="26">
+        <f>SUM(F2:F23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>Adafruit parts shaded and sorted first (preferred supplier). Non-Adafruit parts have no Adafruit equivalent. Prices 2026-07-05: 'VERIFIED' seen in a distributor listing this session; 'ESTIMATE' from prior knowledge/typical range - confirm before ordering. Unit prices (blue) editable; totals are formulas.</t>
         </is>

</xml_diff>